<commit_message>
Add final changes before switching
</commit_message>
<xml_diff>
--- a/resources/template.xlsx
+++ b/resources/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/iestyngage/git/LabelTransaction/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21082F1-DA73-594D-ACAF-DCD321CE485C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA37B8F-F5CF-6F47-B826-5334A0A4F63E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1500" windowWidth="27240" windowHeight="15560" xr2:uid="{CDBF9494-2178-B143-8977-F3547BA7C8A8}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16780" xr2:uid="{CDBF9494-2178-B143-8977-F3547BA7C8A8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -73,12 +73,6 @@
     <t>Food</t>
   </si>
   <si>
-    <t>Rewards</t>
-  </si>
-  <si>
-    <t>Car</t>
-  </si>
-  <si>
     <t>Refunds</t>
   </si>
   <si>
@@ -97,18 +91,9 @@
     <t>Entertainment</t>
   </si>
   <si>
-    <t>Investing</t>
-  </si>
-  <si>
-    <t>Savings</t>
-  </si>
-  <si>
     <t>Subscriptions</t>
   </si>
   <si>
-    <t>Charity</t>
-  </si>
-  <si>
     <t>Total of sums</t>
   </si>
   <si>
@@ -119,6 +104,21 @@
   </si>
   <si>
     <t>Holiday</t>
+  </si>
+  <si>
+    <t>Bank cashback</t>
+  </si>
+  <si>
+    <t>Bill spliting</t>
+  </si>
+  <si>
+    <t>Additional income</t>
+  </si>
+  <si>
+    <t>Investing &amp; Saving</t>
+  </si>
+  <si>
+    <t>Charity &amp; membership</t>
   </si>
 </sst>
 </file>
@@ -177,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -187,6 +187,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,6 +508,7 @@
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="1.83203125" customWidth="1"/>
     <col min="8" max="8" width="1.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="1.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -534,10 +536,10 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>7</v>
@@ -576,7 +578,7 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <f ca="1">SUM(INDIRECT("E3:E"&amp;ROWS(E:E)))</f>
+        <f ca="1">SUM(INDIRECT("F3:F"&amp;ROWS(F:F)))</f>
         <v>0</v>
       </c>
       <c r="I3" t="s">
@@ -595,10 +597,10 @@
         <v>5</v>
       </c>
       <c r="I4" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="J4">
-        <f t="shared" ref="J4:J6" si="0">SUMIF($O:$O,I4,$N:$N)</f>
+        <f t="shared" ref="J4:J8" si="0">SUMIF($O:$O,I4,$N:$N)</f>
         <v>0</v>
       </c>
     </row>
@@ -610,9 +612,9 @@
         <f t="shared" ref="B5:B18" si="1">SUMIF($G:$G,A5,$F:$F)</f>
         <v>0</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="5"/>
       <c r="I5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J5">
         <f t="shared" si="0"/>
@@ -628,7 +630,7 @@
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J6">
         <f t="shared" si="0"/>
@@ -643,13 +645,27 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="I7" t="s">
+        <v>25</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8">
         <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="I8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -673,7 +689,7 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B11">
         <f t="shared" si="1"/>
@@ -682,7 +698,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B12">
         <f t="shared" si="1"/>
@@ -691,7 +707,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B13">
         <f t="shared" si="1"/>
@@ -700,7 +716,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B14">
         <f t="shared" si="1"/>
@@ -718,30 +734,18 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B16">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ref="B16" si="2">SUMIF($G:$G,A16,$F:$F)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>